<commit_message>
review(vol4 ch12): repair AI prose and rescue continuity; sync reading copies and final audit table
</commit_message>
<xml_diff>
--- a/08-审稿/章节最终审核总表.xlsx
+++ b/08-审稿/章节最终审核总表.xlsx
@@ -57,7 +57,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Z13"/>
+  <dimension ref="A1:Z25"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -1497,7 +1497,1303 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="21" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>第004章</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>脏雪与热汤</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第086章.md</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>e9219c9dbd2cec5c205edcaffc15a23da2e227af</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第004章-独立正文质量审查与修订-20261101.md</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I14" s="2">
+        <v>76.5</v>
+      </c>
+      <c r="J14" s="2">
+        <v>82.5</v>
+      </c>
+      <c r="K14" s="2">
+        <v>6</v>
+      </c>
+      <c r="L14" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="M14" s="2">
+        <v>7.8</v>
+      </c>
+      <c r="N14" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="O14" s="2">
+        <v>8.6</v>
+      </c>
+      <c r="P14" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="R14" s="2">
+        <v>7.9</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T14" s="2">
+        <v>23</v>
+      </c>
+      <c r="U14" s="2">
+        <v>0</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>GitHub端定向同步；本地Python脚本与XLSX未验收</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>已同步；与正文转换一致</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>定向第004章已同步；全量脚本未执行</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>单模型反证</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="21" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>第010章</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>没人愿意签的撤兵令</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第092章.md</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ea3153ad47ee75175728f044d0e081de7c033ae2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第010章-独立正文质量审查与复验-20261101.md</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I15" s="2">
+        <v>71.3</v>
+      </c>
+      <c r="J15" s="2">
+        <v>79.9</v>
+      </c>
+      <c r="K15" s="2">
+        <v>8.6</v>
+      </c>
+      <c r="L15" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="M15" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="N15" s="2">
+        <v>7.6</v>
+      </c>
+      <c r="O15" s="2">
+        <v>8</v>
+      </c>
+      <c r="P15" s="2">
+        <v>7.8</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="R15" s="2">
+        <v>7.7</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T15" s="2">
+        <v>28</v>
+      </c>
+      <c r="U15" s="2">
+        <v>0</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>GitHub端定向TXT及合订本校验；正式Python及全卷验收未执行</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>按导出逻辑同步、源文逐字符核对</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>目标章节条目同步、全卷脚本未执行</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>单模型反证</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="21" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>第018章</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>被钉在布告栏的人</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第100章.md</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>9b62b0a5ba50514075ef95ac1a6915dd270f815f</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第018章-独立正文质量审查与复验-20261101.md</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I16" s="2">
+        <v>69.1</v>
+      </c>
+      <c r="J16" s="2">
+        <v>79.6</v>
+      </c>
+      <c r="K16" s="2">
+        <v>10.5</v>
+      </c>
+      <c r="L16" s="2">
+        <v>7.9</v>
+      </c>
+      <c r="M16" s="2">
+        <v>7.9</v>
+      </c>
+      <c r="N16" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="O16" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="P16" s="2">
+        <v>7.9</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>7.7</v>
+      </c>
+      <c r="R16" s="2">
+        <v>7.9</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T16" s="2">
+        <v>54</v>
+      </c>
+      <c r="U16" s="2">
+        <v>0</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>GitHub端定向同步一致；正式Python/XLSX未验收</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>按正式转换逻辑同步</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>目标章唯一替换；未运行全卷脚本</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>单模型反证</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="21" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>第017章</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>江小年的证词</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第099章.md</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>f01a097de7aebe2adc6ef38832f7b5013b2af721</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第017章-独立正文质量审查与修订-20261101.md</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I17" s="2">
+        <v>76.4</v>
+      </c>
+      <c r="J17" s="2">
+        <v>81.4</v>
+      </c>
+      <c r="K17" s="2">
+        <v>5</v>
+      </c>
+      <c r="L17" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="M17" s="2">
+        <v>8</v>
+      </c>
+      <c r="N17" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="O17" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="P17" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="R17" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T17" s="2">
+        <v>91</v>
+      </c>
+      <c r="U17" s="2">
+        <v>0</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>GitHub端定向文本核对；官方Python/XLSX未验收</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>目标章等值转换已核对</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>第017章条目定向同步；全量脚本未运行</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>单模型反证</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>第013章（全书095）</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>只有四声应答</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第095章.md</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>f24e4200d376fec237f3ec34156ec7fa0d826ce0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第013章-独立正文质量审查与复验-20261101.md</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I18" s="2">
+        <v>77.1</v>
+      </c>
+      <c r="J18" s="2">
+        <v>83.1</v>
+      </c>
+      <c r="K18" s="2">
+        <v>6</v>
+      </c>
+      <c r="L18" s="2">
+        <v>8.6</v>
+      </c>
+      <c r="M18" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="N18" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="O18" s="2">
+        <v>8.5</v>
+      </c>
+      <c r="P18" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>8</v>
+      </c>
+      <c r="R18" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T18" s="2">
+        <v>31</v>
+      </c>
+      <c r="U18" s="2">
+        <v>0</v>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>GitHub定向同规则转换通过；正式Python及XLSX未校验</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>MD转换等值通过</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>只更新第013章并核对边界；官方--all --check未执行</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>单模型反证</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="21" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>第016章（全书第098章）</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>一个没接通的信标</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第098章.md</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>cbca667bc36d862d52815b76df7fd54385dbe0fa</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第016章-独立正文质量审查与复验-20261101.md</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I19" s="2">
+        <v>75.5</v>
+      </c>
+      <c r="J19" s="2">
+        <v>80.5</v>
+      </c>
+      <c r="K19" s="2">
+        <v>5</v>
+      </c>
+      <c r="L19" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="M19" s="2">
+        <v>8</v>
+      </c>
+      <c r="N19" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="O19" s="2">
+        <v>8</v>
+      </c>
+      <c r="P19" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>8</v>
+      </c>
+      <c r="R19" s="2">
+        <v>8</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T19" s="2">
+        <v>30</v>
+      </c>
+      <c r="U19" s="2">
+        <v>0</v>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>GitHub端按脚本文本逻辑定向同步；正式Python/XLSX未验收</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>定向等值</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>合订本第016章条目定向等值，未全卷校验</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>单模型反证</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="21" customHeight="1">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>第019章</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>你见过他救人</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第101章.md</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>c9bc50c518bc6c0fea831c5ed329383bdb3939e4</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第019章-独立正文质量审查与复验-20261101.md</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I20" s="2">
+        <v>76.3</v>
+      </c>
+      <c r="J20" s="2">
+        <v>82.3</v>
+      </c>
+      <c r="K20" s="2">
+        <v>6</v>
+      </c>
+      <c r="L20" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="M20" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="N20" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="O20" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="P20" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="R20" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T20" s="2">
+        <v>48</v>
+      </c>
+      <c r="U20" s="2">
+        <v>0</v>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>GitHub端定向文本已核对；正式Python及XLSX未验收</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>脚本等价转换逐字核对</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>仅本章条目定向替换；未跑全卷校验</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>单模型反证</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="21" customHeight="1">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>第014章</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>阵亡表的空白</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第096章.md</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>539dca97541ead5f9eab828575146a088638f94a</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第014章-独立正文质量审查与修订-20261101.md</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I21" s="2">
+        <v>71.3</v>
+      </c>
+      <c r="J21" s="2">
+        <v>82.4</v>
+      </c>
+      <c r="K21" s="2">
+        <v>11.1</v>
+      </c>
+      <c r="L21" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="M21" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="N21" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="O21" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="P21" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>8.4</v>
+      </c>
+      <c r="R21" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T21" s="2">
+        <v>32</v>
+      </c>
+      <c r="U21" s="2">
+        <v>0</v>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>工程部分完成：定向同步；正式Python/XLSX未验收</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>已同步；GitHub回读与正文导出一致</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>仅本章区块更新，全卷脚本未跑</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>单模型隔离反证</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="21" customHeight="1">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>第015章</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>钢臂里的编号</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第097章.md</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>9b62b0a5ba50514075ef95ac1a6915dd270f815f</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第015章-独立正文质量审查与修订-20261101.md</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I22" s="2">
+        <v>74.5</v>
+      </c>
+      <c r="J22" s="2">
+        <v>80.9</v>
+      </c>
+      <c r="K22" s="2">
+        <v>6.4</v>
+      </c>
+      <c r="L22" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="M22" s="2">
+        <v>7.8</v>
+      </c>
+      <c r="N22" s="2">
+        <v>8.4</v>
+      </c>
+      <c r="O22" s="2">
+        <v>8</v>
+      </c>
+      <c r="P22" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>8</v>
+      </c>
+      <c r="R22" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T22" s="2">
+        <v>35</v>
+      </c>
+      <c r="U22" s="2">
+        <v>0</v>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>未完全验收：本地脚本及XLSX待同步</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>GitHub定向同步；官方脚本未运行</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>GitHub定向同步；官方全量校验未运行</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>单模型反证</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="21" customHeight="1">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>第011章（全书第093章）</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>西侧缺口</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第093章.md</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>a53375befe46842e5c51bd31c664e496722713da</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第011章-独立正文质量审查与复验-20261101.md</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I23" s="2">
+        <v>76.3</v>
+      </c>
+      <c r="J23" s="2">
+        <v>81.7</v>
+      </c>
+      <c r="K23" s="2">
+        <v>5.4</v>
+      </c>
+      <c r="L23" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="M23" s="2">
+        <v>8</v>
+      </c>
+      <c r="N23" s="2">
+        <v>8</v>
+      </c>
+      <c r="O23" s="2">
+        <v>8.4</v>
+      </c>
+      <c r="P23" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="R23" s="2">
+        <v>8.5</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T23" s="2">
+        <v>32</v>
+      </c>
+      <c r="U23" s="2">
+        <v>0</v>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>GitHub端等价文本核验；正式Python/XLSX未验收</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>MD-TXT等价转换逐字一致</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>合订本第011章条目唯一替换；未运行正式全卷校验</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>单模型反证</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="21" customHeight="1">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>第020章（全书第102章）</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>灰雀的证物袋</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第102章.md</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>源blob:dac67ed34d5c466566f121337f94f468b4c4cc11</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第020章-独立正文质量审查与修订-20261101.md</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I24" s="2">
+        <v>70.2</v>
+      </c>
+      <c r="J24" s="2">
+        <v>80.7</v>
+      </c>
+      <c r="K24" s="2">
+        <v>10.5</v>
+      </c>
+      <c r="L24" s="2">
+        <v>8</v>
+      </c>
+      <c r="M24" s="2">
+        <v>8</v>
+      </c>
+      <c r="N24" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="O24" s="2">
+        <v>8.3</v>
+      </c>
+      <c r="P24" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="R24" s="2">
+        <v>7.9</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T24" s="2">
+        <v>38</v>
+      </c>
+      <c r="U24" s="2">
+        <v>0</v>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>GitHub文本比对;正式Python/XLSX未验收</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>定向转换一致;需--check</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>定向020和021同步;需全量脚本检查</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>单模型反证</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="21" customHeight="1">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>崖边戍卒</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>第四卷</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>第012章</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>铁砧最后一次接应</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>06-正文/第四卷/第094章.md</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>ad7abc9c6ee1b53e8b27c70f83dbb422966e123c</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>08-审稿/第四卷第012章-独立正文质量审查与复验-20261101.md</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I25" s="2">
+        <v>69.7</v>
+      </c>
+      <c r="J25" s="2">
+        <v>81.9</v>
+      </c>
+      <c r="K25" s="2">
+        <v>12.2</v>
+      </c>
+      <c r="L25" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="M25" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="N25" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="O25" s="2">
+        <v>8.5</v>
+      </c>
+      <c r="P25" s="2">
+        <v>8.2</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>8</v>
+      </c>
+      <c r="R25" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="T25" s="2">
+        <v>31</v>
+      </c>
+      <c r="U25" s="2">
+        <v>0</v>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>GitHub定向等价校验；正式Python脚本未执行</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>MD/TXT按转换规则吻合</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>第012/013章合订条目唯一，正式全卷检查未执行</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>单模型反证（降级）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z13"/>
+  <autoFilter ref="A1:Z25"/>
 </worksheet>
 </file>
</xml_diff>